<commit_message>
first block is done
</commit_message>
<xml_diff>
--- a/Data/data_four_species.xlsx
+++ b/Data/data_four_species.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\OneDrive\Рабочий стол\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7446033E-3379-447C-B1B4-54F402EBADFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A53F024-DF00-49F1-9FCD-01EEF20193F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Fluke_data" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="fluke_data" sheetId="1" r:id="rId1"/>
+    <sheet name="liver_data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -145,18 +145,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -458,1006 +451,1006 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>0</v>
-      </c>
-      <c r="F7" s="10">
-        <v>0</v>
-      </c>
-      <c r="G7" s="10">
+      <c r="C7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+      <c r="A8">
         <v>2</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
-      <c r="F8" s="8">
-        <v>0</v>
-      </c>
-      <c r="G8" s="8">
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0</v>
-      </c>
-      <c r="F9" s="8">
-        <v>0</v>
-      </c>
-      <c r="G9" s="8">
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>4</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0</v>
-      </c>
-      <c r="F10" s="8">
-        <v>0</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
-        <v>5</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="A11" s="1">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="2">
+      <c r="C11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="1">
         <v>1</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>0.8</v>
       </c>
-      <c r="F11" s="9">
-        <v>0</v>
-      </c>
-      <c r="G11" s="9">
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+      <c r="A12" s="2">
         <v>1</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="3">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3">
-        <v>0</v>
-      </c>
-      <c r="F12" s="10">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10">
-        <v>0</v>
-      </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
+      <c r="C12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
+      <c r="A13">
         <v>2</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0</v>
-      </c>
-      <c r="F13" s="8">
-        <v>0</v>
-      </c>
-      <c r="G13" s="8">
-        <v>0</v>
-      </c>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
-        <v>3</v>
-      </c>
-      <c r="B14" s="1" t="s">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0</v>
-      </c>
-      <c r="E14" s="1">
-        <v>0</v>
-      </c>
-      <c r="F14" s="8">
-        <v>5</v>
-      </c>
-      <c r="G14" s="8">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>5</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
-        <v>4</v>
-      </c>
-      <c r="B15" s="1" t="s">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D15" s="1">
-        <v>0</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
-      <c r="F15" s="8">
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
         <v>25</v>
       </c>
-      <c r="G15" s="8">
-        <v>0</v>
-      </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
-        <v>5</v>
-      </c>
-      <c r="B16" s="2" t="s">
+      <c r="A16" s="1">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D16" s="2">
+      <c r="C16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="1">
         <v>1</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>0.7</v>
       </c>
-      <c r="F16" s="9">
-        <v>0</v>
-      </c>
-      <c r="G16" s="9">
-        <v>0</v>
-      </c>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="3">
+      <c r="A17" s="2">
         <v>1</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D17" s="3">
+      <c r="C17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2">
         <v>22</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="2">
         <v>3.4</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="5">
         <v>110</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="5">
         <v>2.8</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
+      <c r="A18">
         <v>2</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D18" s="4">
+      <c r="C18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18">
         <v>24</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18">
         <v>3.5</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="3">
         <v>120</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="3">
         <v>4.5</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
-        <v>3</v>
-      </c>
-      <c r="B19" s="1" t="s">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D19" s="4">
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19">
         <v>24</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19">
         <v>3.6</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="3">
         <v>130</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
-        <v>4</v>
-      </c>
-      <c r="B20" s="1" t="s">
+      <c r="A20">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
         <v>8</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="4">
+      <c r="C20" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20">
         <v>25</v>
       </c>
-      <c r="E20" s="1">
-        <v>4</v>
-      </c>
-      <c r="F20" s="8">
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20" s="3">
         <v>140</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="3">
         <v>6.4</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
-        <v>5</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="A21" s="1">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="2">
+      <c r="C21" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="1">
         <v>27</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>5.7</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="4">
         <v>200</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
+      <c r="A22">
         <v>1</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="4">
-        <v>0</v>
-      </c>
-      <c r="E22" s="4">
-        <v>0</v>
-      </c>
-      <c r="F22" s="8">
-        <v>0</v>
-      </c>
-      <c r="G22" s="8">
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
+      <c r="A23">
         <v>2</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="4">
-        <v>0</v>
-      </c>
-      <c r="E23" s="4">
-        <v>0</v>
-      </c>
-      <c r="F23" s="8">
-        <v>0</v>
-      </c>
-      <c r="G23" s="8">
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
-        <v>3</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="4">
-        <v>0</v>
-      </c>
-      <c r="E24" s="4">
-        <v>0</v>
-      </c>
-      <c r="F24" s="8">
-        <v>0</v>
-      </c>
-      <c r="G24" s="8">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
-        <v>4</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="4">
-        <v>0</v>
-      </c>
-      <c r="E25" s="4">
-        <v>0</v>
-      </c>
-      <c r="F25" s="8">
-        <v>0</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="A25">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>5</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="5">
-        <v>0</v>
-      </c>
-      <c r="E26" s="5">
-        <v>0</v>
-      </c>
-      <c r="F26" s="9">
-        <v>0</v>
-      </c>
-      <c r="G26" s="9">
+      <c r="A26" s="1">
+        <v>5</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="3">
+      <c r="A27" s="2">
         <v>1</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="3">
-        <v>0</v>
-      </c>
-      <c r="E27" s="3">
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2">
         <v>0.2</v>
       </c>
-      <c r="F27" s="10">
-        <v>0</v>
-      </c>
-      <c r="G27" s="8">
+      <c r="F27" s="5">
+        <v>0</v>
+      </c>
+      <c r="G27" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
+      <c r="A28">
         <v>2</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>6</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="1">
+      <c r="C28" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28">
         <v>1</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28">
         <v>0.7</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="3">
         <v>180</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="1">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="A29">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="1">
+      <c r="C29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29">
         <v>1</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29">
         <v>0.9</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="3">
         <v>220</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="1">
-        <v>4</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="A30">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="1">
+      <c r="C30" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30">
         <v>2</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30">
         <v>1.4</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="3">
         <v>80</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="3">
         <v>0.2</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="2">
-        <v>5</v>
-      </c>
-      <c r="B31" s="2" t="s">
+      <c r="A31" s="1">
+        <v>5</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="2">
-        <v>3</v>
-      </c>
-      <c r="E31" s="2">
+      <c r="C31" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="1">
+        <v>3</v>
+      </c>
+      <c r="E31" s="1">
         <v>1.9</v>
       </c>
-      <c r="F31" s="9">
+      <c r="F31" s="4">
         <v>99</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="4">
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="1">
+      <c r="A32">
         <v>1</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="4">
-        <v>3</v>
-      </c>
-      <c r="E32" s="1">
+      <c r="C32" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32">
+        <v>3</v>
+      </c>
+      <c r="E32">
         <v>0.8</v>
       </c>
-      <c r="F32" s="8">
-        <v>0</v>
-      </c>
-      <c r="G32" s="10">
+      <c r="F32" s="3">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="1">
+      <c r="A33">
         <v>2</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="4">
-        <v>5</v>
-      </c>
-      <c r="E33" s="1">
+      <c r="C33" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33">
         <v>0.9</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="3">
         <v>35</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
-        <v>3</v>
-      </c>
-      <c r="B34" s="1" t="s">
+      <c r="A34">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="4">
+      <c r="C34" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34">
         <v>7</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34">
         <v>3.9</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="3">
         <v>60</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="1">
-        <v>4</v>
-      </c>
-      <c r="B35" s="1" t="s">
+      <c r="A35">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="4">
+      <c r="C35" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35">
         <v>9</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35">
         <v>6</v>
       </c>
-      <c r="F35" s="8">
-        <v>0</v>
-      </c>
-      <c r="G35" s="8">
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="2">
-        <v>5</v>
-      </c>
-      <c r="B36" s="2" t="s">
+      <c r="A36" s="1">
+        <v>5</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D36" s="5">
+      <c r="C36" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="1">
         <v>14</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>7</v>
       </c>
-      <c r="F36" s="9">
+      <c r="F36" s="4">
         <v>19</v>
       </c>
-      <c r="G36" s="9">
+      <c r="G36" s="4">
         <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="3">
+      <c r="A37" s="2">
         <v>1</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" s="6">
+      <c r="C37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2">
         <v>32</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E37" s="2">
         <v>3.8</v>
       </c>
-      <c r="F37" s="10">
+      <c r="F37" s="5">
         <v>1050</v>
       </c>
-      <c r="G37" s="10">
+      <c r="G37" s="5">
         <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
+      <c r="A38">
         <v>2</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>8</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="4">
+      <c r="C38" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38">
         <v>35</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38">
         <v>4.5</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="3">
         <v>1200</v>
       </c>
-      <c r="G38" s="8">
+      <c r="G38" s="3">
         <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
-        <v>3</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="A39">
+        <v>3</v>
+      </c>
+      <c r="B39" t="s">
         <v>8</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D39" s="4">
+      <c r="C39" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39">
         <v>36</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39">
         <v>4.7</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="3">
         <v>1250</v>
       </c>
-      <c r="G39" s="8">
+      <c r="G39" s="3">
         <v>33</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
-        <v>4</v>
-      </c>
-      <c r="B40" s="1" t="s">
+      <c r="A40">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="4">
+      <c r="C40" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40">
         <v>44</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40">
         <v>5.2</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F40" s="3">
         <v>1400</v>
       </c>
-      <c r="G40" s="8">
+      <c r="G40" s="3">
         <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="2">
-        <v>5</v>
-      </c>
-      <c r="B41" s="2" t="s">
+      <c r="A41" s="1">
+        <v>5</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D41" s="5">
+      <c r="C41" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="1">
         <v>49</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41" s="1">
         <v>5.6</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="4">
         <v>1650</v>
       </c>
-      <c r="G41" s="9">
+      <c r="G41" s="4">
         <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="G45" s="7"/>
-      <c r="H45" s="7"/>
-      <c r="I45" s="7"/>
-      <c r="J45" s="7"/>
-      <c r="K45" s="7"/>
-      <c r="L45" s="7"/>
-      <c r="M45" s="7"/>
-      <c r="N45" s="7"/>
-      <c r="O45" s="7"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
-      <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
-      <c r="L46" s="7"/>
-      <c r="M46" s="7"/>
-      <c r="N46" s="7"/>
-      <c r="O46" s="7"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="7"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
-      <c r="L47" s="7"/>
-      <c r="M47" s="7"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="7"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="G48" s="7"/>
-      <c r="H48" s="7"/>
-      <c r="I48" s="7"/>
-      <c r="J48" s="7"/>
-      <c r="K48" s="7"/>
-      <c r="L48" s="7"/>
-      <c r="M48" s="7"/>
-      <c r="N48" s="7"/>
-      <c r="O48" s="7"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1513,19 +1506,19 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2">
         <v>0.1</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2">
         <v>0.1</v>
       </c>
       <c r="F2">
@@ -1534,27 +1527,27 @@
       <c r="G2">
         <v>0</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2">
         <v>13</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>0.4</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
@@ -1563,27 +1556,27 @@
       <c r="G3">
         <v>0.2</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3">
         <v>18</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>0.5</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>0.2</v>
       </c>
       <c r="F4">
@@ -1592,27 +1585,27 @@
       <c r="G4">
         <v>0.2</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4">
         <v>21</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>0.7</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5">
         <v>0.3</v>
       </c>
       <c r="F5">
@@ -1621,27 +1614,27 @@
       <c r="G5">
         <v>0.4</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5">
         <v>21</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>0.9</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>0.5</v>
       </c>
       <c r="F6">
@@ -1650,27 +1643,27 @@
       <c r="G6">
         <v>0.6</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>23</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3">
+      <c r="B7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
         <v>0.4</v>
       </c>
       <c r="F7">
@@ -1679,27 +1672,27 @@
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <v>20</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="2">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+      <c r="A8">
         <v>2</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D8" s="1">
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8">
         <v>0.1</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8">
         <v>0.5</v>
       </c>
       <c r="F8">
@@ -1708,27 +1701,27 @@
       <c r="G8">
         <v>0.1</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8">
         <v>21</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D9" s="1">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9">
         <v>0.2</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9">
         <v>0.5</v>
       </c>
       <c r="F9">
@@ -1737,27 +1730,27 @@
       <c r="G9">
         <v>0.2</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9">
         <v>22</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9">
         <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>4</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="1">
+      <c r="A10">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10">
         <v>0.3</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10">
         <v>0.7</v>
       </c>
       <c r="F10">
@@ -1766,27 +1759,27 @@
       <c r="G10">
         <v>0.4</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10">
         <v>22</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
-        <v>5</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="2">
+      <c r="A11" s="1">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="1">
         <v>0.4</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>0.9</v>
       </c>
       <c r="F11">
@@ -1795,27 +1788,27 @@
       <c r="G11">
         <v>0.2</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>23</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+      <c r="A12" s="2">
         <v>1</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="3">
+      <c r="B12" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2">
         <v>0.2</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="2">
         <v>0.2</v>
       </c>
       <c r="F12">
@@ -1824,27 +1817,27 @@
       <c r="G12">
         <v>0</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="2">
         <v>21</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="2">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
+      <c r="A13">
         <v>2</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="1">
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13">
         <v>0.3</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13">
         <v>0.3</v>
       </c>
       <c r="F13">
@@ -1853,27 +1846,27 @@
       <c r="G13">
         <v>0.1</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13">
         <v>21</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13">
         <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
-        <v>3</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" s="1">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14">
         <v>0.4</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14">
         <v>0.4</v>
       </c>
       <c r="F14">
@@ -1882,27 +1875,27 @@
       <c r="G14">
         <v>0.1</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14">
         <v>22</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
-        <v>4</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="1">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15">
         <v>0.6</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15">
         <v>0.6</v>
       </c>
       <c r="F15">
@@ -1911,27 +1904,27 @@
       <c r="G15">
         <v>0.2</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15">
         <v>24</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
-        <v>5</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="2">
+      <c r="A16" s="1">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="1">
         <v>0.8</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>0.9</v>
       </c>
       <c r="F16">
@@ -1940,27 +1933,27 @@
       <c r="G16">
         <v>0.3</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>25</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="3">
+      <c r="A17" s="2">
         <v>1</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>0.1</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="2">
         <v>0</v>
       </c>
       <c r="F17">
@@ -1969,27 +1962,27 @@
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="2">
         <v>19</v>
       </c>
-      <c r="I17" s="3">
+      <c r="I17" s="2">
         <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
+      <c r="A18">
         <v>2</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18">
         <v>0.2</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
@@ -1998,27 +1991,27 @@
       <c r="G18">
         <v>0.2</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18">
         <v>21</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18">
         <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
-        <v>3</v>
-      </c>
-      <c r="B19" s="1" t="s">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19">
         <v>0.4</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
@@ -2027,27 +2020,27 @@
       <c r="G19">
         <v>0.3</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19">
         <v>23</v>
       </c>
-      <c r="I19" s="1">
+      <c r="I19">
         <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
-        <v>4</v>
-      </c>
-      <c r="B20" s="1" t="s">
+      <c r="A20">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20">
         <v>0.8</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20">
         <v>0.2</v>
       </c>
       <c r="F20">
@@ -2056,27 +2049,27 @@
       <c r="G20">
         <v>0.3</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20">
         <v>23</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20">
         <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
-        <v>5</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="A21" s="1">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>2</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>2</v>
       </c>
       <c r="F21">
@@ -2085,27 +2078,27 @@
       <c r="G21">
         <v>0.5</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>24</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="1">
         <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="3">
+      <c r="A22" s="2">
         <v>1</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22" s="3">
-        <v>3</v>
-      </c>
-      <c r="E22" s="3">
+      <c r="C22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="2">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2">
         <v>3</v>
       </c>
       <c r="F22">
@@ -2114,27 +2107,27 @@
       <c r="G22">
         <v>3</v>
       </c>
-      <c r="H22" s="3">
+      <c r="H22" s="2">
         <v>31</v>
       </c>
-      <c r="I22" s="3">
+      <c r="I22" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
+      <c r="A23">
         <v>2</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="1">
+      <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23">
         <v>3.2</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23">
         <v>3.6</v>
       </c>
       <c r="F23">
@@ -2143,27 +2136,27 @@
       <c r="G23">
         <v>4.2</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23">
         <v>32</v>
       </c>
-      <c r="I23" s="1">
+      <c r="I23">
         <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
-        <v>3</v>
-      </c>
-      <c r="B24" s="1" t="s">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="1">
+      <c r="C24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24">
         <v>4.0999999999999996</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24">
         <v>4.7</v>
       </c>
       <c r="F24">
@@ -2172,27 +2165,27 @@
       <c r="G24">
         <v>5.5</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24">
         <v>33</v>
       </c>
-      <c r="I24" s="1">
+      <c r="I24">
         <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
-        <v>4</v>
-      </c>
-      <c r="B25" s="1" t="s">
+      <c r="A25">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="1">
+      <c r="C25" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25">
         <v>4.5</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25">
         <v>5</v>
       </c>
       <c r="F25">
@@ -2201,27 +2194,27 @@
       <c r="G25">
         <v>6.3</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25">
         <v>33</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25">
         <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>5</v>
-      </c>
-      <c r="B26" s="2" t="s">
+      <c r="A26" s="1">
+        <v>5</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D26" s="2">
+      <c r="C26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="1">
         <v>9.3000000000000007</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>6.2</v>
       </c>
       <c r="F26">
@@ -2230,27 +2223,27 @@
       <c r="G26">
         <v>9.6</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>34</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26" s="1">
         <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="3">
+      <c r="A27" s="2">
         <v>1</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="3">
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2">
         <v>3.4</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27" s="2">
         <v>3.7</v>
       </c>
       <c r="F27">
@@ -2259,27 +2252,27 @@
       <c r="G27">
         <v>1.8</v>
       </c>
-      <c r="H27" s="3">
+      <c r="H27" s="2">
         <v>30</v>
       </c>
-      <c r="I27" s="3">
+      <c r="I27" s="2">
         <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
+      <c r="A28">
         <v>2</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>6</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="1">
+      <c r="C28" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28">
         <v>5.2</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E28">
         <v>3.8</v>
       </c>
       <c r="F28">
@@ -2288,27 +2281,27 @@
       <c r="G28">
         <v>2.5</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28">
         <v>31</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28">
         <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="1">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="A29">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="1">
+      <c r="C29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29">
         <v>5.6</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29">
         <v>3.9</v>
       </c>
       <c r="F29">
@@ -2317,27 +2310,27 @@
       <c r="G29">
         <v>3.2</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29">
         <v>31</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29">
         <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="1">
-        <v>4</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="A30">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="1">
+      <c r="C30" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30">
         <v>5.9</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E30">
         <v>7.2</v>
       </c>
       <c r="F30">
@@ -2346,27 +2339,27 @@
       <c r="G30">
         <v>4</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30">
         <v>32</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30">
         <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="2">
-        <v>5</v>
-      </c>
-      <c r="B31" s="2" t="s">
+      <c r="A31" s="1">
+        <v>5</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="2">
+      <c r="C31" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="1">
         <v>9.4</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>13.2</v>
       </c>
       <c r="F31">
@@ -2375,27 +2368,27 @@
       <c r="G31">
         <v>10</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>33</v>
       </c>
-      <c r="I31" s="2">
+      <c r="I31" s="1">
         <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="3">
+      <c r="A32" s="2">
         <v>1</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="3">
-        <v>0</v>
-      </c>
-      <c r="E32" s="3">
+      <c r="D32" s="2">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2">
         <v>0</v>
       </c>
       <c r="F32">
@@ -2404,27 +2397,27 @@
       <c r="G32">
         <v>0</v>
       </c>
-      <c r="H32" s="3">
+      <c r="H32" s="2">
         <v>20</v>
       </c>
-      <c r="I32" s="3">
+      <c r="I32" s="2">
         <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="1">
+      <c r="A33">
         <v>2</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" t="s">
         <v>14</v>
       </c>
-      <c r="D33" s="1">
-        <v>0</v>
-      </c>
-      <c r="E33" s="1">
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
         <v>0</v>
       </c>
       <c r="F33">
@@ -2433,27 +2426,27 @@
       <c r="G33">
         <v>0</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33">
         <v>22</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33">
         <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
-        <v>3</v>
-      </c>
-      <c r="B34" s="1" t="s">
+      <c r="A34">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" t="s">
         <v>14</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34">
         <v>0.1</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34">
         <v>0.1</v>
       </c>
       <c r="F34">
@@ -2462,27 +2455,27 @@
       <c r="G34">
         <v>0</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34">
         <v>22</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34">
         <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="1">
-        <v>4</v>
-      </c>
-      <c r="B35" s="1" t="s">
+      <c r="A35">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35">
         <v>0.1</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35">
         <v>0.1</v>
       </c>
       <c r="F35">
@@ -2491,27 +2484,27 @@
       <c r="G35">
         <v>0.2</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35">
         <v>24</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35">
         <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="2">
-        <v>5</v>
-      </c>
-      <c r="B36" s="2" t="s">
+      <c r="A36" s="1">
+        <v>5</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>0.2</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>0.1</v>
       </c>
       <c r="F36">
@@ -2520,27 +2513,27 @@
       <c r="G36">
         <v>0.4</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>28</v>
       </c>
-      <c r="I36" s="2">
+      <c r="I36" s="1">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="3">
+      <c r="A37" s="2">
         <v>1</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D37" s="3">
-        <v>0</v>
-      </c>
-      <c r="E37" s="3">
+      <c r="C37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="2">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2">
         <v>0.2</v>
       </c>
       <c r="F37">
@@ -2549,27 +2542,27 @@
       <c r="G37">
         <v>0.8</v>
       </c>
-      <c r="H37" s="3">
+      <c r="H37" s="2">
         <v>32</v>
       </c>
-      <c r="I37" s="3">
+      <c r="I37" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
+      <c r="A38">
         <v>2</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D38" s="1">
+      <c r="C38" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38">
         <v>1.8</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38">
         <v>1.5</v>
       </c>
       <c r="F38">
@@ -2578,27 +2571,27 @@
       <c r="G38">
         <v>1.8</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38">
         <v>38</v>
       </c>
-      <c r="I38" s="1">
+      <c r="I38">
         <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
-        <v>3</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="A39">
+        <v>3</v>
+      </c>
+      <c r="B39" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D39" s="1">
+      <c r="C39" t="s">
+        <v>4</v>
+      </c>
+      <c r="D39">
         <v>5.7</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39">
         <v>1.8</v>
       </c>
       <c r="F39">
@@ -2607,27 +2600,27 @@
       <c r="G39">
         <v>2</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39">
         <v>42</v>
       </c>
-      <c r="I39" s="1">
+      <c r="I39">
         <v>12</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
-        <v>4</v>
-      </c>
-      <c r="B40" s="1" t="s">
+      <c r="A40">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
         <v>7</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D40" s="1">
+      <c r="C40" t="s">
+        <v>4</v>
+      </c>
+      <c r="D40">
         <v>6.9</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40">
         <v>2.1</v>
       </c>
       <c r="F40">
@@ -2636,27 +2629,27 @@
       <c r="G40">
         <v>2.2999999999999998</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40">
         <v>43</v>
       </c>
-      <c r="I40" s="1">
+      <c r="I40">
         <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="2">
-        <v>5</v>
-      </c>
-      <c r="B41" s="2" t="s">
+      <c r="A41" s="1">
+        <v>5</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D41" s="2">
+      <c r="C41" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D41" s="1">
         <v>7</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41" s="1">
         <v>7.4</v>
       </c>
       <c r="F41">
@@ -2665,27 +2658,27 @@
       <c r="G41">
         <v>4.5</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46</v>
       </c>
-      <c r="I41" s="2">
+      <c r="I41" s="1">
         <v>19</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="3">
+      <c r="A42" s="2">
         <v>1</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D42" s="3">
+      <c r="C42" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="2">
         <v>1.3</v>
       </c>
-      <c r="E42" s="3">
+      <c r="E42" s="2">
         <v>1.3</v>
       </c>
       <c r="F42">
@@ -2694,27 +2687,27 @@
       <c r="G42">
         <v>1</v>
       </c>
-      <c r="H42" s="3">
+      <c r="H42" s="2">
         <v>30</v>
       </c>
-      <c r="I42" s="3">
+      <c r="I42" s="2">
         <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
+      <c r="A43">
         <v>2</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>7</v>
       </c>
-      <c r="C43" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D43" s="1">
+      <c r="C43" t="s">
+        <v>5</v>
+      </c>
+      <c r="D43">
         <v>2.6</v>
       </c>
-      <c r="E43" s="1">
+      <c r="E43">
         <v>1.4</v>
       </c>
       <c r="F43">
@@ -2723,27 +2716,27 @@
       <c r="G43">
         <v>1.5</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43">
         <v>35</v>
       </c>
-      <c r="I43" s="1">
+      <c r="I43">
         <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="1">
-        <v>3</v>
-      </c>
-      <c r="B44" s="1" t="s">
+      <c r="A44">
+        <v>3</v>
+      </c>
+      <c r="B44" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D44" s="1">
+      <c r="C44" t="s">
+        <v>5</v>
+      </c>
+      <c r="D44">
         <v>3.1</v>
       </c>
-      <c r="E44" s="1">
+      <c r="E44">
         <v>0.5</v>
       </c>
       <c r="F44">
@@ -2752,27 +2745,27 @@
       <c r="G44">
         <v>5</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44">
         <v>36</v>
       </c>
-      <c r="I44" s="1">
+      <c r="I44">
         <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" s="1">
-        <v>4</v>
-      </c>
-      <c r="B45" s="1" t="s">
+      <c r="A45">
+        <v>4</v>
+      </c>
+      <c r="B45" t="s">
         <v>7</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D45" s="1">
+      <c r="C45" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45">
         <v>6</v>
       </c>
-      <c r="E45" s="1">
+      <c r="E45">
         <v>4.8</v>
       </c>
       <c r="F45">
@@ -2781,27 +2774,27 @@
       <c r="G45">
         <v>10</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45">
         <v>37</v>
       </c>
-      <c r="I45" s="1">
+      <c r="I45">
         <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="2">
-        <v>5</v>
-      </c>
-      <c r="B46" s="2" t="s">
+      <c r="A46" s="1">
+        <v>5</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D46" s="2">
+      <c r="C46" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D46" s="1">
         <v>12.7</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E46" s="1">
         <v>14</v>
       </c>
       <c r="F46">
@@ -2810,27 +2803,27 @@
       <c r="G46">
         <v>24</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>42</v>
       </c>
-      <c r="I46" s="2">
+      <c r="I46" s="1">
         <v>34</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="3">
+      <c r="A47" s="2">
         <v>1</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D47" s="3">
+      <c r="D47" s="2">
         <v>0.1</v>
       </c>
-      <c r="E47" s="3">
+      <c r="E47" s="2">
         <v>0</v>
       </c>
       <c r="F47">
@@ -2839,27 +2832,27 @@
       <c r="G47">
         <v>0</v>
       </c>
-      <c r="H47" s="3">
+      <c r="H47" s="2">
         <v>10</v>
       </c>
-      <c r="I47" s="3">
+      <c r="I47" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="1">
+      <c r="A48">
         <v>2</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>8</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" t="s">
         <v>14</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48">
         <v>0.2</v>
       </c>
-      <c r="E48" s="1">
+      <c r="E48">
         <v>0</v>
       </c>
       <c r="F48">
@@ -2868,27 +2861,27 @@
       <c r="G48">
         <v>0</v>
       </c>
-      <c r="H48" s="1">
+      <c r="H48">
         <v>12</v>
       </c>
-      <c r="I48" s="1">
+      <c r="I48">
         <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="1">
-        <v>3</v>
-      </c>
-      <c r="B49" s="1" t="s">
+      <c r="A49">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s">
         <v>8</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" t="s">
         <v>14</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49">
         <v>0.2</v>
       </c>
-      <c r="E49" s="1">
+      <c r="E49">
         <v>0.1</v>
       </c>
       <c r="F49">
@@ -2897,27 +2890,27 @@
       <c r="G49">
         <v>0</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49">
         <v>14</v>
       </c>
-      <c r="I49" s="1">
+      <c r="I49">
         <v>12</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" s="1">
-        <v>4</v>
-      </c>
-      <c r="B50" s="1" t="s">
+      <c r="A50">
+        <v>4</v>
+      </c>
+      <c r="B50" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" t="s">
         <v>14</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50">
         <v>0.4</v>
       </c>
-      <c r="E50" s="1">
+      <c r="E50">
         <v>0.1</v>
       </c>
       <c r="F50">
@@ -2926,27 +2919,27 @@
       <c r="G50">
         <v>0.1</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50">
         <v>18</v>
       </c>
-      <c r="I50" s="1">
+      <c r="I50">
         <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="2">
-        <v>5</v>
-      </c>
-      <c r="B51" s="2" t="s">
+      <c r="A51" s="1">
+        <v>5</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>0.6</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E51" s="1">
         <v>0.3</v>
       </c>
       <c r="F51">
@@ -2955,27 +2948,27 @@
       <c r="G51">
         <v>0.2</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>16</v>
       </c>
-      <c r="I51" s="2">
+      <c r="I51" s="1">
         <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="3">
+      <c r="A52" s="2">
         <v>1</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D52" s="3">
+      <c r="C52" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" s="2">
         <v>6.2</v>
       </c>
-      <c r="E52" s="3">
+      <c r="E52" s="2">
         <v>3.9</v>
       </c>
       <c r="F52">
@@ -2984,27 +2977,27 @@
       <c r="G52">
         <v>9</v>
       </c>
-      <c r="H52" s="3">
+      <c r="H52" s="2">
         <v>18</v>
       </c>
-      <c r="I52" s="3">
+      <c r="I52" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" s="1">
+      <c r="A53">
         <v>2</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>8</v>
       </c>
-      <c r="C53" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D53" s="1">
+      <c r="C53" t="s">
+        <v>4</v>
+      </c>
+      <c r="D53">
         <v>6.5</v>
       </c>
-      <c r="E53" s="1">
+      <c r="E53">
         <v>6.3</v>
       </c>
       <c r="F53">
@@ -3013,27 +3006,27 @@
       <c r="G53">
         <v>13.5</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53">
         <v>19</v>
       </c>
-      <c r="I53" s="1">
+      <c r="I53">
         <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" s="1">
-        <v>3</v>
-      </c>
-      <c r="B54" s="1" t="s">
+      <c r="A54">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
         <v>8</v>
       </c>
-      <c r="C54" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D54" s="1">
+      <c r="C54" t="s">
+        <v>4</v>
+      </c>
+      <c r="D54">
         <v>6.8</v>
       </c>
-      <c r="E54" s="1">
+      <c r="E54">
         <v>6.7</v>
       </c>
       <c r="F54">
@@ -3042,27 +3035,27 @@
       <c r="G54">
         <v>15</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54">
         <v>20</v>
       </c>
-      <c r="I54" s="1">
+      <c r="I54">
         <v>14</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="1">
-        <v>4</v>
-      </c>
-      <c r="B55" s="1" t="s">
+      <c r="A55">
+        <v>4</v>
+      </c>
+      <c r="B55" t="s">
         <v>8</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D55" s="1">
+      <c r="C55" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55">
         <v>7.4</v>
       </c>
-      <c r="E55" s="1">
+      <c r="E55">
         <v>8.3000000000000007</v>
       </c>
       <c r="F55">
@@ -3071,27 +3064,27 @@
       <c r="G55">
         <v>17.5</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55">
         <v>20</v>
       </c>
-      <c r="I55" s="1">
+      <c r="I55">
         <v>20</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="2">
-        <v>5</v>
-      </c>
-      <c r="B56" s="2" t="s">
+      <c r="A56" s="1">
+        <v>5</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C56" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D56" s="2">
+      <c r="C56" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="1">
         <v>8</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>11.2</v>
       </c>
       <c r="F56">
@@ -3100,27 +3093,27 @@
       <c r="G56">
         <v>20</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>21</v>
       </c>
-      <c r="I56" s="2">
+      <c r="I56" s="1">
         <v>20</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="3">
+      <c r="A57" s="2">
         <v>1</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B57" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D57" s="3">
+      <c r="C57" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D57" s="2">
         <v>6.3</v>
       </c>
-      <c r="E57" s="3">
+      <c r="E57" s="2">
         <v>8.1999999999999993</v>
       </c>
       <c r="F57">
@@ -3129,27 +3122,27 @@
       <c r="G57">
         <v>5</v>
       </c>
-      <c r="H57" s="3">
+      <c r="H57" s="2">
         <v>37</v>
       </c>
-      <c r="I57" s="3">
+      <c r="I57" s="2">
         <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="1">
+      <c r="A58">
         <v>2</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>8</v>
       </c>
-      <c r="C58" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D58" s="1">
+      <c r="C58" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58">
         <v>7.8</v>
       </c>
-      <c r="E58" s="1">
+      <c r="E58">
         <v>10.3</v>
       </c>
       <c r="F58">
@@ -3158,27 +3151,27 @@
       <c r="G58">
         <v>9</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58">
         <v>49</v>
       </c>
-      <c r="I58" s="1">
+      <c r="I58">
         <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="1">
-        <v>3</v>
-      </c>
-      <c r="B59" s="1" t="s">
+      <c r="A59">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s">
         <v>8</v>
       </c>
-      <c r="C59" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D59" s="1">
+      <c r="C59" t="s">
+        <v>5</v>
+      </c>
+      <c r="D59">
         <v>8.4</v>
       </c>
-      <c r="E59" s="1">
+      <c r="E59">
         <v>11</v>
       </c>
       <c r="F59">
@@ -3187,27 +3180,27 @@
       <c r="G59">
         <v>12</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59">
         <v>56</v>
       </c>
-      <c r="I59" s="1">
+      <c r="I59">
         <v>67</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="1">
-        <v>4</v>
-      </c>
-      <c r="B60" s="1" t="s">
+      <c r="A60">
+        <v>4</v>
+      </c>
+      <c r="B60" t="s">
         <v>8</v>
       </c>
-      <c r="C60" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D60" s="1">
+      <c r="C60" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60">
         <v>8.8000000000000007</v>
       </c>
-      <c r="E60" s="1">
+      <c r="E60">
         <v>12.5</v>
       </c>
       <c r="F60">
@@ -3216,27 +3209,27 @@
       <c r="G60">
         <v>16</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60">
         <v>52</v>
       </c>
-      <c r="I60" s="1">
+      <c r="I60">
         <v>72</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="2">
-        <v>5</v>
-      </c>
-      <c r="B61" s="2" t="s">
+      <c r="A61" s="1">
+        <v>5</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D61" s="2">
+      <c r="C61" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" s="1">
         <v>9.1999999999999993</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E61" s="1">
         <v>14</v>
       </c>
       <c r="F61">
@@ -3245,10 +3238,10 @@
       <c r="G61">
         <v>18.5</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>57</v>
       </c>
-      <c r="I61" s="2">
+      <c r="I61" s="1">
         <v>76</v>
       </c>
     </row>

</xml_diff>

<commit_message>
boxplots are colored right
</commit_message>
<xml_diff>
--- a/Data/data_four_species.xlsx
+++ b/Data/data_four_species.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\OneDrive\Рабочий стол\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A53F024-DF00-49F1-9FCD-01EEF20193F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6940D9-C1B4-4B01-BEE0-B6AB62F4A18C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15360" yWindow="0" windowWidth="15360" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fluke_data" sheetId="1" r:id="rId1"/>
@@ -1079,7 +1079,7 @@
       <c r="E27" s="2">
         <v>0.2</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="3">
         <v>0</v>
       </c>
       <c r="G27" s="3">
@@ -1103,7 +1103,7 @@
         <v>0.7</v>
       </c>
       <c r="F28" s="3">
-        <v>180</v>
+        <v>35</v>
       </c>
       <c r="G28" s="3">
         <v>0</v>
@@ -1126,7 +1126,7 @@
         <v>0.9</v>
       </c>
       <c r="F29" s="3">
-        <v>220</v>
+        <v>60</v>
       </c>
       <c r="G29" s="3">
         <v>0</v>
@@ -1149,7 +1149,7 @@
         <v>1.4</v>
       </c>
       <c r="F30" s="3">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3">
         <v>0.2</v>
@@ -1172,7 +1172,7 @@
         <v>1.9</v>
       </c>
       <c r="F31" s="4">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="G31" s="4">
         <v>2.2000000000000002</v>
@@ -1194,7 +1194,7 @@
       <c r="E32">
         <v>0.8</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="5">
         <v>0</v>
       </c>
       <c r="G32" s="5">
@@ -1218,7 +1218,7 @@
         <v>0.9</v>
       </c>
       <c r="F33" s="3">
-        <v>35</v>
+        <v>180</v>
       </c>
       <c r="G33" s="3">
         <v>0</v>
@@ -1241,7 +1241,7 @@
         <v>3.9</v>
       </c>
       <c r="F34" s="3">
-        <v>60</v>
+        <v>220</v>
       </c>
       <c r="G34" s="3">
         <v>0</v>
@@ -1264,7 +1264,7 @@
         <v>6</v>
       </c>
       <c r="F35" s="3">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="G35" s="3">
         <v>4</v>
@@ -1287,7 +1287,7 @@
         <v>7</v>
       </c>
       <c r="F36" s="4">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="G36" s="4">
         <v>23</v>

</xml_diff>

<commit_message>
box_plots for histology are done
</commit_message>
<xml_diff>
--- a/Data/data_four_species.xlsx
+++ b/Data/data_four_species.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\OneDrive\Рабочий стол\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6940D9-C1B4-4B01-BEE0-B6AB62F4A18C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73242FF9-AD13-40CC-9A44-DB3EE642D4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15360" yWindow="0" windowWidth="15360" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fluke_data" sheetId="1" r:id="rId1"/>
@@ -1522,7 +1522,7 @@
         <v>0.1</v>
       </c>
       <c r="F2">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1551,7 +1551,7 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="G3">
         <v>0.2</v>
@@ -1580,7 +1580,7 @@
         <v>0.2</v>
       </c>
       <c r="F4">
-        <v>2.2000000000000002</v>
+        <v>0.2</v>
       </c>
       <c r="G4">
         <v>0.2</v>
@@ -1609,7 +1609,7 @@
         <v>0.3</v>
       </c>
       <c r="F5">
-        <v>2.6</v>
+        <v>0.1</v>
       </c>
       <c r="G5">
         <v>0.4</v>
@@ -1638,7 +1638,7 @@
         <v>0.5</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="G6">
         <v>0.6</v>
@@ -1957,7 +1957,7 @@
         <v>0</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>0.2</v>
       </c>
       <c r="G18">
         <v>0.2</v>
@@ -2015,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>0.1</v>
       </c>
       <c r="G19">
         <v>0.3</v>
@@ -2044,7 +2044,7 @@
         <v>0.2</v>
       </c>
       <c r="F20">
-        <v>4.5</v>
+        <v>0.3</v>
       </c>
       <c r="G20">
         <v>0.3</v>
@@ -2073,7 +2073,7 @@
         <v>2</v>
       </c>
       <c r="F21">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G21">
         <v>0.5</v>
@@ -2392,7 +2392,7 @@
         <v>0</v>
       </c>
       <c r="F32">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G32">
         <v>0</v>
@@ -2421,7 +2421,7 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="G33">
         <v>0</v>
@@ -2450,7 +2450,7 @@
         <v>0.1</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="G34">
         <v>0</v>
@@ -2479,7 +2479,7 @@
         <v>0.1</v>
       </c>
       <c r="F35">
-        <v>2.5</v>
+        <v>0.1</v>
       </c>
       <c r="G35">
         <v>0.2</v>
@@ -2508,7 +2508,7 @@
         <v>0.1</v>
       </c>
       <c r="F36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G36">
         <v>0.4</v>
@@ -2827,7 +2827,7 @@
         <v>0</v>
       </c>
       <c r="F47">
-        <v>3.5</v>
+        <v>0.1</v>
       </c>
       <c r="G47">
         <v>0</v>
@@ -2856,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="F48">
-        <v>4</v>
+        <v>0.2</v>
       </c>
       <c r="G48">
         <v>0</v>
@@ -2885,7 +2885,7 @@
         <v>0.1</v>
       </c>
       <c r="F49">
-        <v>4.2</v>
+        <v>0.1</v>
       </c>
       <c r="G49">
         <v>0</v>
@@ -2914,7 +2914,7 @@
         <v>0.1</v>
       </c>
       <c r="F50">
-        <v>4.8</v>
+        <v>0.2</v>
       </c>
       <c r="G50">
         <v>0.1</v>
@@ -2943,7 +2943,7 @@
         <v>0.3</v>
       </c>
       <c r="F51">
-        <v>5.2</v>
+        <v>0.3</v>
       </c>
       <c r="G51">
         <v>0.2</v>

</xml_diff>

<commit_message>
Work is done for today
</commit_message>
<xml_diff>
--- a/Data/data_four_species.xlsx
+++ b/Data/data_four_species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\OneDrive\Рабочий стол\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73242FF9-AD13-40CC-9A44-DB3EE642D4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCF579E-404A-4263-B94A-674BFE7DD557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1524,8 +1524,8 @@
       <c r="F2">
         <v>0.1</v>
       </c>
-      <c r="G2">
-        <v>0</v>
+      <c r="G2" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H2">
         <v>13</v>
@@ -1547,8 +1547,8 @@
       <c r="D3">
         <v>0.4</v>
       </c>
-      <c r="E3">
-        <v>0</v>
+      <c r="E3" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F3">
         <v>0.3</v>
@@ -1661,7 +1661,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="2">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="E7" s="2">
         <v>0.4</v>
@@ -1669,8 +1669,8 @@
       <c r="F7">
         <v>1.8</v>
       </c>
-      <c r="G7">
-        <v>0</v>
+      <c r="G7" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H7" s="2">
         <v>20</v>
@@ -1814,8 +1814,8 @@
       <c r="F12">
         <v>1.8</v>
       </c>
-      <c r="G12">
-        <v>0</v>
+      <c r="G12" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H12" s="2">
         <v>21</v>
@@ -1954,13 +1954,13 @@
         <v>0.1</v>
       </c>
       <c r="E17" s="2">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F17">
         <v>0.1</v>
       </c>
-      <c r="G17">
-        <v>0</v>
+      <c r="G17" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H17" s="2">
         <v>19</v>
@@ -1982,8 +1982,8 @@
       <c r="D18">
         <v>0.2</v>
       </c>
-      <c r="E18">
-        <v>0</v>
+      <c r="E18" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F18">
         <v>0.2</v>
@@ -2011,8 +2011,8 @@
       <c r="D19">
         <v>0.4</v>
       </c>
-      <c r="E19">
-        <v>0</v>
+      <c r="E19" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F19">
         <v>0.1</v>
@@ -2072,8 +2072,8 @@
       <c r="E21" s="1">
         <v>2</v>
       </c>
-      <c r="F21">
-        <v>0</v>
+      <c r="F21" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="G21">
         <v>0.5</v>
@@ -2386,16 +2386,16 @@
         <v>14</v>
       </c>
       <c r="D32" s="2">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="E32" s="2">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F32">
         <v>0.1</v>
       </c>
-      <c r="G32">
-        <v>0</v>
+      <c r="G32" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H32" s="2">
         <v>20</v>
@@ -2414,17 +2414,17 @@
       <c r="C33" t="s">
         <v>14</v>
       </c>
-      <c r="D33">
-        <v>0</v>
-      </c>
-      <c r="E33">
-        <v>0</v>
+      <c r="D33" s="2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="E33" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F33">
         <v>0.2</v>
       </c>
-      <c r="G33">
-        <v>0</v>
+      <c r="G33" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H33">
         <v>22</v>
@@ -2452,8 +2452,8 @@
       <c r="F34">
         <v>0.2</v>
       </c>
-      <c r="G34">
-        <v>0</v>
+      <c r="G34" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H34">
         <v>22</v>
@@ -2507,8 +2507,8 @@
       <c r="E36" s="1">
         <v>0.1</v>
       </c>
-      <c r="F36">
-        <v>0</v>
+      <c r="F36" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="G36">
         <v>0.4</v>
@@ -2531,7 +2531,7 @@
         <v>4</v>
       </c>
       <c r="D37" s="2">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="E37" s="2">
         <v>0.2</v>
@@ -2824,13 +2824,13 @@
         <v>0.1</v>
       </c>
       <c r="E47" s="2">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F47">
         <v>0.1</v>
       </c>
-      <c r="G47">
-        <v>0</v>
+      <c r="G47" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H47" s="2">
         <v>10</v>
@@ -2853,13 +2853,13 @@
         <v>0.2</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="F48">
         <v>0.2</v>
       </c>
-      <c r="G48">
-        <v>0</v>
+      <c r="G48" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H48">
         <v>12</v>
@@ -2887,8 +2887,8 @@
       <c r="F49">
         <v>0.1</v>
       </c>
-      <c r="G49">
-        <v>0</v>
+      <c r="G49" s="2">
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="H49">
         <v>14</v>

</xml_diff>